<commit_message>
``` chore: rename database backup from backup15.sql to backup.sql and update Excel templates
- Renamed backup/backup15.sql to backup.sql and updated all references in db-integrity-rule.md
- Updated Excel templates: CXC.xlsx, CXP.xlsx, ENTRADA ALMACEN.xlsx, and REMISION.xlsx (binary files modified)
- Changed database source of truth documentation from backup15.sql to backup.sql across all validation rules
```
</commit_message>
<xml_diff>
--- a/Excel-templates/CXP.xlsx
+++ b/Excel-templates/CXP.xlsx
@@ -1748,13 +1748,13 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="16" fontId="2" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="17" fontId="12" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -10506,15 +10506,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="129" customFormat="1" ht="19.5" thickBot="1">
-      <c r="A1" s="156" t="s">
+      <c r="A1" s="154" t="s">
         <v>340</v>
       </c>
-      <c r="B1" s="154"/>
-      <c r="C1" s="154"/>
-      <c r="D1" s="154"/>
-      <c r="E1" s="154"/>
-      <c r="F1" s="154"/>
-      <c r="G1" s="154"/>
+      <c r="B1" s="155"/>
+      <c r="C1" s="155"/>
+      <c r="D1" s="155"/>
+      <c r="E1" s="155"/>
+      <c r="F1" s="155"/>
+      <c r="G1" s="155"/>
     </row>
     <row r="2" spans="1:8" s="129" customFormat="1" ht="15.75" thickBot="1">
       <c r="A2" s="111" t="s">
@@ -10744,11 +10744,14 @@
     </row>
     <row r="24" spans="1:9" s="131" customFormat="1" ht="15.75" thickBot="1">
       <c r="A24" s="141"/>
-      <c r="B24" s="155" t="s">
+      <c r="B24" s="156" t="s">
         <v>248</v>
       </c>
-      <c r="C24" s="155"/>
-      <c r="D24" s="142"/>
+      <c r="C24" s="156"/>
+      <c r="D24" s="142">
+        <f>SUM(D4:D23)</f>
+        <v>0</v>
+      </c>
       <c r="E24" s="143"/>
       <c r="F24" s="144"/>
       <c r="G24" s="145"/>
@@ -10778,15 +10781,15 @@
       <c r="I26" s="133"/>
     </row>
     <row r="27" spans="1:9" ht="19.5" thickBot="1">
-      <c r="A27" s="156" t="s">
+      <c r="A27" s="154" t="s">
         <v>339</v>
       </c>
-      <c r="B27" s="154"/>
-      <c r="C27" s="154"/>
-      <c r="D27" s="154"/>
-      <c r="E27" s="154"/>
-      <c r="F27" s="154"/>
-      <c r="G27" s="154"/>
+      <c r="B27" s="155"/>
+      <c r="C27" s="155"/>
+      <c r="D27" s="155"/>
+      <c r="E27" s="155"/>
+      <c r="F27" s="155"/>
+      <c r="G27" s="155"/>
     </row>
     <row r="28" spans="1:9" ht="15.75" thickBot="1">
       <c r="A28" s="111" t="s">
@@ -10970,11 +10973,14 @@
     </row>
     <row r="46" spans="1:9" ht="15.75" thickBot="1">
       <c r="A46" s="141"/>
-      <c r="B46" s="155" t="s">
+      <c r="B46" s="156" t="s">
         <v>248</v>
       </c>
-      <c r="C46" s="155"/>
-      <c r="D46" s="142"/>
+      <c r="C46" s="156"/>
+      <c r="D46" s="142">
+        <f>SUM(D30:D44)</f>
+        <v>0</v>
+      </c>
       <c r="E46" s="143"/>
       <c r="F46" s="144"/>
       <c r="G46" s="145"/>
@@ -11198,11 +11204,14 @@
     </row>
     <row r="70" spans="1:9" s="129" customFormat="1" ht="15.75" thickBot="1">
       <c r="A70" s="141"/>
-      <c r="B70" s="155" t="s">
+      <c r="B70" s="156" t="s">
         <v>248</v>
       </c>
-      <c r="C70" s="155"/>
-      <c r="D70" s="142"/>
+      <c r="C70" s="156"/>
+      <c r="D70" s="142">
+        <f>SUM(D52:D68)</f>
+        <v>0</v>
+      </c>
       <c r="E70" s="143"/>
       <c r="F70" s="144"/>
       <c r="G70" s="145"/>

</xml_diff>